<commit_message>
summary of all the spectral models attempted
</commit_message>
<xml_diff>
--- a/xray_epoch_spec_models.xlsx
+++ b/xray_epoch_spec_models.xlsx
@@ -1,40 +1,145 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adeutsch/SN2018ivc_2026/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AE5D6F-FF3F-984D-9B0C-F1EC70DC9E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="9060" yWindow="820" windowWidth="20080" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="bestmodel" sheetId="1" r:id="rId1"/>
+    <sheet name="allmodelsummary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+  <si>
+    <t>Epoch</t>
+  </si>
+  <si>
+    <t>Best Model</t>
+  </si>
+  <si>
+    <t>rstat or wstat</t>
+  </si>
+  <si>
+    <t>powerlaw, with n_H frozen to galactic, since thawing it didn't help.</t>
+  </si>
+  <si>
+    <t>29071+29072</t>
+  </si>
+  <si>
+    <t>powerlaw alone, N_H frozen to galactic. Switched 2026-09-08 from bremss+powerlaw: all models fit statistically indistinguishably well here (rstat&lt;=0.2), but bremss+powerlaw's 2 extra free params are degenerate at only 109 counts (thermal/nonthermal trade off freely), giving a huge one-sided flux/luminosity error (~800x the median). Powerlaw alone is well-constrained (Gamma=1.33+/-0.19, ~20% norm error) and gives a usable luminosity error bar (~13%).</t>
+  </si>
+  <si>
+    <t>31211+31996</t>
+  </si>
+  <si>
+    <t>bremss+free gaussian (E=2.957+/-0.032, \sigma=0.055 keV, res limit). width hits energy resolution floor, indicating line narrower than observation resolution</t>
+  </si>
+  <si>
+    <t>1.15, \Delta W = 9.50</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Frozen Params</t>
+  </si>
+  <si>
+    <t>Free Params</t>
+  </si>
+  <si>
+    <t>Physical Interpretation</t>
+  </si>
+  <si>
+    <t>apec</t>
+  </si>
+  <si>
+    <t>powerlaw</t>
+  </si>
+  <si>
+    <t>bremss</t>
+  </si>
+  <si>
+    <t>abundance (Z=solar), redshift (z=0.003793)</t>
+  </si>
+  <si>
+    <t>all models multiplied by tbabs, frozen to n_H=2.6*10^20 cm^-2, galactic</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>photon index (\Gamma), normalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plasma temperature (kT), normalization </t>
+  </si>
+  <si>
+    <t>Functional Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">none, interpolated from a grid of models from the ATOMDB atomic database </t>
+  </si>
+  <si>
+    <t>collisionally ionized thermal plasma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">free-free emission, single T thermal plasm </t>
+  </si>
+  <si>
+    <t>nonthermal: synchrotron, IC</t>
+  </si>
+  <si>
+    <t>KE^{-\Gamma}</t>
+  </si>
+  <si>
+    <t>\propto \frac{K}{\sqrt{T}}g(E,T)\exp{-E/kT}E^{-1}</t>
+  </si>
+  <si>
+    <t>bremss+powerlaw</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="20"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <color theme="1"/>
-      <sz val="20"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,82 +157,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -447,80 +494,155 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="27" x14ac:dyDescent="0.35"/>
   <cols>
-    <col width="22.5" customWidth="1" style="1" min="1" max="1"/>
-    <col width="102.6640625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="19.83203125" customWidth="1" style="1" min="3" max="3"/>
-    <col width="10.83203125" customWidth="1" style="1" min="4" max="16384"/>
+    <col min="1" max="1" width="22.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="102.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Epoch</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Best Model</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>rstat or wstat</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
         <v>20306</v>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>powerlaw, with n_H frozen to galactic, since thawing it didn't help.</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
         <v>2.27</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>29071+29072</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>powerlaw alone, N_H frozen to galactic. Switched 2026-09-08 from bremss+powerlaw: all models fit statistically indistinguishably well here (rstat&lt;=0.2), but bremss+powerlaw's 2 extra free params are degenerate at only 109 counts (thermal/nonthermal trade off freely), giving a huge one-sided flux/luminosity error (~800x the median). Powerlaw alone is well-constrained (Gamma=1.33+/-0.19, ~20% norm error) and gives a usable luminosity error bar (~13%).</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
         <v>0.17</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>31211+31996</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>bremss+free gaussian (E=2.957+/-0.032, \sigma=0.055 keV, res limit). width hits energy resolution floor, indicating line narrower than observation resolution</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>1.15, \Delta W = 9.50</t>
-        </is>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75FDE4E4-E663-6440-ACFB-4475AA318130}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="24" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="56.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="51.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="62.33203125" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>